<commit_message>
feat: allow the user to select the seat reservation officers
</commit_message>
<xml_diff>
--- a/samples/ra/26-27/Royal Arch Official Visit Matrix 2026 - 2027 MF V7 26082026.xlsx
+++ b/samples/ra/26-27/Royal Arch Official Visit Matrix 2026 - 2027 MF V7 26082026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kpturner/github/square_ov/samples/ra/26-27/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD5EAAC3-5EF9-FD4A-AEB6-FD693CB626F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A83DF413-A9EE-7D43-A9FA-A4263278E8B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="47900" windowHeight="22920" tabRatio="500" activeTab="1" xr2:uid="{FA0C5B21-D744-41D8-A854-64181BC35FE8}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="47900" windowHeight="22920" tabRatio="500" xr2:uid="{FA0C5B21-D744-41D8-A854-64181BC35FE8}"/>
   </bookViews>
   <sheets>
     <sheet name="2026-2027 Official Visits" sheetId="1" r:id="rId1"/>
@@ -71,7 +71,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1523" uniqueCount="575">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1517" uniqueCount="569">
   <si>
     <t>Name</t>
   </si>
@@ -1756,15 +1756,6 @@
     <t>103 Station Rd, Drayton, Portsmouth PO6 1PL</t>
   </si>
   <si>
-    <t>Charles</t>
-  </si>
-  <si>
-    <t>McGeoch</t>
-  </si>
-  <si>
-    <t>PProvGSE</t>
-  </si>
-  <si>
     <t>Jordan</t>
   </si>
   <si>
@@ -1817,15 +1808,6 @@
   </si>
   <si>
     <t>n.sharifi@yahoo.co.uk</t>
-  </si>
-  <si>
-    <t>Past Provincial Grand Scribe E</t>
-  </si>
-  <si>
-    <t>MCGEOCH</t>
-  </si>
-  <si>
-    <t>charles@mcgeoch.com</t>
   </si>
 </sst>
 </file>
@@ -4295,7 +4277,7 @@
         <v>141</v>
       </c>
       <c r="AE3" s="210" t="s">
-        <v>562</v>
+        <v>559</v>
       </c>
       <c r="AF3" s="51" t="s">
         <v>142</v>
@@ -8805,7 +8787,7 @@
         <v>8</v>
       </c>
       <c r="F54" s="130" t="s">
-        <v>561</v>
+        <v>558</v>
       </c>
       <c r="G54" s="21" t="s">
         <v>510</v>
@@ -9060,13 +9042,13 @@
         <v>159</v>
       </c>
       <c r="B57" s="208" t="s">
-        <v>551</v>
+        <v>200</v>
       </c>
       <c r="C57" s="76" t="s">
-        <v>552</v>
-      </c>
-      <c r="D57" s="76" t="s">
-        <v>553</v>
+        <v>175</v>
+      </c>
+      <c r="D57" s="4" t="s">
+        <v>98</v>
       </c>
       <c r="E57" s="43">
         <f t="shared" si="4"/>
@@ -9122,7 +9104,7 @@
       </c>
       <c r="AO57" s="12" t="str">
         <f t="shared" si="6"/>
-        <v>Charles McGeoch</v>
+        <v>Gifton Roy Bailey</v>
       </c>
     </row>
     <row r="58" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.15">
@@ -9135,7 +9117,7 @@
       <c r="C58" s="72" t="s">
         <v>116</v>
       </c>
-      <c r="D58" s="72" t="s">
+      <c r="D58" s="4" t="s">
         <v>98</v>
       </c>
       <c r="E58" s="73">
@@ -9210,7 +9192,7 @@
         <v>520</v>
       </c>
       <c r="D59" s="26" t="s">
-        <v>559</v>
+        <v>556</v>
       </c>
       <c r="E59" s="43">
         <f t="shared" si="4"/>
@@ -9280,13 +9262,13 @@
         <v>162</v>
       </c>
       <c r="B60" s="26" t="s">
-        <v>554</v>
+        <v>551</v>
       </c>
       <c r="C60" s="26" t="s">
         <v>40</v>
       </c>
       <c r="D60" s="26" t="s">
-        <v>555</v>
+        <v>552</v>
       </c>
       <c r="E60" s="43">
         <f t="shared" si="4"/>
@@ -9358,13 +9340,13 @@
         <v>163</v>
       </c>
       <c r="B61" s="26" t="s">
-        <v>556</v>
+        <v>553</v>
       </c>
       <c r="C61" s="27" t="s">
-        <v>557</v>
+        <v>554</v>
       </c>
       <c r="D61" s="26" t="s">
-        <v>558</v>
+        <v>555</v>
       </c>
       <c r="E61" s="43">
         <f t="shared" si="4"/>
@@ -9516,7 +9498,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{208D5B5F-72B6-4B46-BC27-C77853048EC1}">
-  <dimension ref="D3:S60"/>
+  <dimension ref="D3:S59"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="4" max="4" width="45.5" style="122" bestFit="1" customWidth="1"/>
@@ -9592,7 +9574,7 @@
         <v>535</v>
       </c>
       <c r="N4" s="216" t="s">
-        <v>560</v>
+        <v>557</v>
       </c>
     </row>
     <row r="5" spans="4:19" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -11128,18 +11110,18 @@
     </row>
     <row r="51" spans="4:14" ht="15" x14ac:dyDescent="0.15">
       <c r="D51" s="217" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="E51" s="218" t="s">
         <v>519</v>
       </c>
       <c r="F51" s="218" t="s">
-        <v>564</v>
+        <v>561</v>
       </c>
       <c r="G51" s="218"/>
       <c r="H51" s="218"/>
       <c r="I51" s="218" t="s">
-        <v>565</v>
+        <v>562</v>
       </c>
       <c r="J51" s="191" t="s">
         <v>232</v>
@@ -11147,16 +11129,16 @@
       <c r="K51" s="218"/>
       <c r="L51" s="218"/>
       <c r="M51" s="219" t="s">
-        <v>566</v>
+        <v>563</v>
       </c>
       <c r="N51" s="218"/>
     </row>
     <row r="52" spans="4:14" ht="15" x14ac:dyDescent="0.15">
       <c r="D52" s="217" t="s">
-        <v>567</v>
+        <v>564</v>
       </c>
       <c r="E52" s="218" t="s">
-        <v>554</v>
+        <v>551</v>
       </c>
       <c r="F52" s="218" t="s">
         <v>528</v>
@@ -11164,7 +11146,7 @@
       <c r="G52" s="218"/>
       <c r="H52" s="218"/>
       <c r="I52" s="218" t="s">
-        <v>554</v>
+        <v>551</v>
       </c>
       <c r="J52" s="191" t="s">
         <v>232</v>
@@ -11172,24 +11154,24 @@
       <c r="K52" s="218"/>
       <c r="L52" s="218"/>
       <c r="M52" s="219" t="s">
-        <v>568</v>
+        <v>565</v>
       </c>
       <c r="N52" s="218"/>
     </row>
     <row r="53" spans="4:14" ht="15" x14ac:dyDescent="0.15">
       <c r="D53" s="217" t="s">
-        <v>569</v>
+        <v>566</v>
       </c>
       <c r="E53" s="218" t="s">
-        <v>556</v>
+        <v>553</v>
       </c>
       <c r="F53" s="218" t="s">
-        <v>570</v>
+        <v>567</v>
       </c>
       <c r="G53" s="218"/>
       <c r="H53" s="218"/>
       <c r="I53" s="218" t="s">
-        <v>556</v>
+        <v>553</v>
       </c>
       <c r="J53" s="191" t="s">
         <v>232</v>
@@ -11197,34 +11179,21 @@
       <c r="K53" s="218"/>
       <c r="L53" s="218"/>
       <c r="M53" s="219" t="s">
-        <v>571</v>
+        <v>568</v>
       </c>
       <c r="N53" s="218"/>
     </row>
-    <row r="54" spans="4:14" ht="15" x14ac:dyDescent="0.15">
-      <c r="D54" s="217" t="s">
-        <v>572</v>
-      </c>
-      <c r="E54" s="218" t="s">
-        <v>551</v>
-      </c>
-      <c r="F54" s="218" t="s">
-        <v>573</v>
-      </c>
-      <c r="G54" s="218"/>
-      <c r="H54" s="218"/>
-      <c r="I54" s="218" t="s">
-        <v>551</v>
-      </c>
-      <c r="J54" s="191" t="s">
-        <v>232</v>
-      </c>
-      <c r="K54" s="218"/>
-      <c r="L54" s="218"/>
-      <c r="M54" s="219" t="s">
-        <v>574</v>
-      </c>
-      <c r="N54" s="218"/>
+    <row r="54" spans="4:14" x14ac:dyDescent="0.15">
+      <c r="E54" s="115"/>
+      <c r="F54" s="115"/>
+      <c r="G54" s="115"/>
+      <c r="H54" s="115"/>
+      <c r="I54" s="115"/>
+      <c r="J54" s="115"/>
+      <c r="K54" s="115"/>
+      <c r="L54" s="115"/>
+      <c r="M54" s="115"/>
+      <c r="N54" s="115"/>
     </row>
     <row r="55" spans="4:14" x14ac:dyDescent="0.15">
       <c r="E55" s="115"/>
@@ -11286,18 +11255,6 @@
       <c r="M59" s="115"/>
       <c r="N59" s="115"/>
     </row>
-    <row r="60" spans="4:14" x14ac:dyDescent="0.15">
-      <c r="E60" s="115"/>
-      <c r="F60" s="115"/>
-      <c r="G60" s="115"/>
-      <c r="H60" s="115"/>
-      <c r="I60" s="115"/>
-      <c r="J60" s="115"/>
-      <c r="K60" s="115"/>
-      <c r="L60" s="115"/>
-      <c r="M60" s="115"/>
-      <c r="N60" s="115"/>
-    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="M24" r:id="rId1" xr:uid="{32827D19-F359-4B6E-BD34-5C3E3A039AB4}"/>
@@ -11306,12 +11263,11 @@
     <hyperlink ref="M7" r:id="rId4" xr:uid="{003440DB-2110-47D1-87EB-0C39243CEF52}"/>
     <hyperlink ref="M5" r:id="rId5" xr:uid="{463BDF5C-06C6-4A6E-801C-EB42D9FE65B8}"/>
     <hyperlink ref="M6" r:id="rId6" xr:uid="{B9BE327F-0B0E-438C-AB64-1560A36E0C39}"/>
-    <hyperlink ref="M54" r:id="rId7" xr:uid="{B4BF8772-30C2-DC48-AF8E-6FD6B2F74385}"/>
-    <hyperlink ref="M51" r:id="rId8" xr:uid="{AED2E48A-CC0A-8A47-B26F-090C6BAD6142}"/>
-    <hyperlink ref="M53" r:id="rId9" xr:uid="{CDFDA878-B292-434A-BDBF-DE1707FC804A}"/>
-    <hyperlink ref="M52" r:id="rId10" xr:uid="{EE35CCFB-3073-3D41-8498-00F04B926FE6}"/>
+    <hyperlink ref="M51" r:id="rId7" xr:uid="{AED2E48A-CC0A-8A47-B26F-090C6BAD6142}"/>
+    <hyperlink ref="M53" r:id="rId8" xr:uid="{CDFDA878-B292-434A-BDBF-DE1707FC804A}"/>
+    <hyperlink ref="M52" r:id="rId9" xr:uid="{EE35CCFB-3073-3D41-8498-00F04B926FE6}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="8" orientation="landscape" horizontalDpi="0" verticalDpi="0" r:id="rId11"/>
+  <pageSetup paperSize="8" orientation="landscape" horizontalDpi="0" verticalDpi="0" r:id="rId10"/>
 </worksheet>
 </file>
</xml_diff>